<commit_message>
Site updated: 2026-10-22 20:29:35
</commit_message>
<xml_diff>
--- a/material/PPPoECodes.xlsx
+++ b/material/PPPoECodes.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\blog_source\blog\source\material\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Blog\blog_source\blog\source\material\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25714" windowHeight="14477"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25710" windowHeight="14475"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -386,10 +386,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>←客户端指明服务器名称</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>←服务器说明自己的名称</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -571,6 +567,10 @@
   </si>
   <si>
     <t>↑仅后面的数据总长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>←客户端需要的服务类型</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -732,31 +732,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -766,6 +742,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1271,143 +1271,143 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O44"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.25" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="15" width="9.53515625" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.23046875" style="1"/>
+    <col min="1" max="15" width="9.5" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.25" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.15">
+      <c r="A1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7" t="s">
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="7"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N1" s="11"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7" t="s">
+      <c r="D2" s="11"/>
+      <c r="E2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="7"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="F2" s="11"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.15">
+      <c r="A3" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="E3" s="12" t="s">
+      <c r="B3" s="15"/>
+      <c r="E3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="H3" s="9" t="s">
+      <c r="F3" s="15"/>
+      <c r="H3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="10"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H5" s="7" t="s">
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="14"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.15">
+      <c r="H5" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="I5" s="7"/>
+      <c r="I5" s="11"/>
       <c r="J5" s="2" t="s">
         <v>48</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="L5" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="O5" s="11"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.15">
+      <c r="L6" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="O5" s="7"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="L6" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.15">
+      <c r="A8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7" t="s">
+      <c r="D8" s="11"/>
+      <c r="E8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.15">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1421,48 +1421,48 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="7"/>
+      <c r="C11" s="11"/>
       <c r="E11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="7"/>
+      <c r="G11" s="11"/>
       <c r="I11" s="2" t="s">
         <v>38</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="L11" s="8" t="s">
+      <c r="L11" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="7"/>
+      <c r="C12" s="11"/>
       <c r="E12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="7"/>
+      <c r="G12" s="11"/>
       <c r="I12" s="2" t="s">
         <v>39</v>
       </c>
@@ -1472,26 +1472,26 @@
       <c r="L12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M12" s="7" t="s">
+      <c r="M12" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N12" s="7"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N12" s="11"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="7"/>
+      <c r="C13" s="11"/>
       <c r="E13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="7"/>
+      <c r="G13" s="11"/>
       <c r="I13" s="2" t="s">
         <v>40</v>
       </c>
@@ -1501,19 +1501,19 @@
       <c r="L13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M13" s="7" t="s">
+      <c r="M13" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="N13" s="7"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N13" s="11"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="7"/>
+      <c r="C14" s="11"/>
       <c r="I14" s="2" t="s">
         <v>41</v>
       </c>
@@ -1523,19 +1523,19 @@
       <c r="L14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="M14" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="N14" s="7"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N14" s="11"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="7"/>
+      <c r="C15" s="11"/>
       <c r="I15" s="2" t="s">
         <v>42</v>
       </c>
@@ -1545,322 +1545,322 @@
       <c r="L15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M15" s="7" t="s">
+      <c r="M15" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="N15" s="7"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N15" s="11"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="7"/>
+      <c r="C16" s="11"/>
       <c r="L16" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="M16" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="N16" s="7"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N16" s="11"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A17" s="1" t="s">
         <v>76</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="M17" s="7" t="s">
+      <c r="M17" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="N17" s="7"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N17" s="11"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C18" s="7"/>
+      <c r="C18" s="11"/>
       <c r="H18" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="J18" s="7"/>
+      <c r="I18" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="J18" s="11"/>
       <c r="L18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="M18" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="N18" s="7"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N18" s="11"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A19" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="C19" s="7"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="5" t="s">
-        <v>90</v>
+        <v>136</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="J19" s="7"/>
+      <c r="I19" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="J19" s="11"/>
       <c r="L19" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M19" s="7" t="s">
+      <c r="M19" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="N19" s="7"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N19" s="11"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="7"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="J20" s="7"/>
-      <c r="L20" s="8" t="s">
+      <c r="I20" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="J20" s="11"/>
+      <c r="L20" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J21" s="7"/>
+      <c r="I21" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="J21" s="11"/>
       <c r="L21" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="M21" s="7" t="s">
+      <c r="M21" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N21" s="7"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N21" s="11"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="7"/>
+      <c r="B22" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="11"/>
       <c r="H22" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="J22" s="7"/>
+        <v>121</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" s="11"/>
       <c r="L22" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M22" s="7" t="s">
+      <c r="M22" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="N22" s="7"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N22" s="11"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="7"/>
+      <c r="B23" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" s="11"/>
       <c r="H23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="J23" s="7"/>
+      <c r="I23" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="J23" s="11"/>
       <c r="L23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="M23" s="7" t="s">
+      <c r="M23" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="N23" s="7"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N23" s="11"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="C24" s="7"/>
+      <c r="B24" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="11"/>
       <c r="H24" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="J24" s="7"/>
-      <c r="L24" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="J24" s="11"/>
+      <c r="L24" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C25" s="7"/>
+      <c r="B25" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" s="11"/>
       <c r="L25" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M25" s="9" t="s">
+      <c r="M25" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="N25" s="10"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N25" s="14"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A26" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C26" s="7"/>
+      <c r="B26" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="11"/>
       <c r="H26" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M26" s="9" t="s">
+      <c r="M26" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="N26" s="10"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N26" s="14"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.15">
       <c r="H27" s="2" t="s">
         <v>52</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="M27" s="9" t="s">
+      <c r="M27" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="N27" s="10"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N27" s="14"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A28" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H28" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="A29" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="H29" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="I29" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="L28" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="H29" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M29" s="9" t="s">
+      <c r="M29" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="N29" s="10"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="B30" s="13" t="s">
+      <c r="N29" s="14"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="A30" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="B30" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
       <c r="L30" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M30" s="9" t="s">
+      <c r="M30" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="N30" s="10"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N30" s="14"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A31" s="3"/>
       <c r="B31" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -1869,89 +1869,89 @@
       <c r="L31" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="M31" s="9" t="s">
+      <c r="M31" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="N31" s="10"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
+      <c r="N31" s="14"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="A32" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
       <c r="L32" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M32" s="9" t="s">
+      <c r="M32" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="N32" s="10"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="13" t="s">
+      <c r="N32" s="14"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A33" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A34" s="3"/>
       <c r="B34" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="15" t="s">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A35" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A36" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A37" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B37" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="13" t="s">
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A38" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1959,70 +1959,115 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="15" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A39" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
-      <c r="F39" s="15"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B40" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A41" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="14" t="s">
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A42" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A43" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="18"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="17" t="s">
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A44" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="F43" s="16"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>120</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="L28:N28"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="M32:N32"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="H3:O3"/>
     <mergeCell ref="H5:I5"/>
@@ -2039,56 +2084,11 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="F13:G13"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="L20:N20"/>
-    <mergeCell ref="L24:N24"/>
-    <mergeCell ref="L28:N28"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>